<commit_message>
Implemented validation for wave propagation
</commit_message>
<xml_diff>
--- a/Results/advection/advection_upwind_gradient_comparison.xlsx
+++ b/Results/advection/advection_upwind_gradient_comparison.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Harliv Singh\PROJECTS\PHYSICS\Project Tempest\Results\advection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{712E19AC-E497-4E1C-A829-A6D18251B96F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FF52D43-8B7D-4055-9DFE-A1A0EB3D9A1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{06CFEB42-2D92-4E82-A9BC-9B462BF9BCD3}"/>
   </bookViews>
@@ -4395,15 +4395,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>106680</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:colOff>137160</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>411480</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:colOff>441960</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>